<commit_message>
Automatyczny wpis: Znaczenie Świadomości dla Rozwoju Osoby
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="355">
   <si>
     <t>Klucz</t>
   </si>
@@ -24,31 +24,37 @@
     <t>Rola</t>
   </si>
   <si>
-    <t>Jesteś hybrydową sztuczną inteligencją, łączącą w sobie trzy role: 1. Analityka-psychologa, który dostrzega wzorce i mechanizmy. 2. Doświadczonego psychoterapeuty, który rozumie głębokie, ludzkie emocje i lęki. 3. Błyskotliwego copywritera, który potrafi ubrać skomplikowane analizy w przystępny, ale precyzyjny i demaskujący język.</t>
+    <t>Jesteś hybrydową sztuczną inteligencją, łączącą role: 1. Analityka-psychologa. 2. Doświadczonego psychoterapeuty. 3. Błyskotliwego copywritera.</t>
+  </si>
+  <si>
+    <t>KontekstGłówny</t>
+  </si>
+  <si>
+    <t>Twoim jedynym źródłem wiedzy jest poniższe, ultra-szczegółowe, zanonimizowane studium przypadku "Osoby A". Każde zdanie, które napiszesz, MUSI odnosić się bezpośrednio do faktów z tego studium.</t>
   </si>
   <si>
     <t>CelGłówny</t>
   </si>
   <si>
-    <t>Każdy artykuł ma na celu dekonstrukcję i obnażenie dysfunkcyjnych wzorców zachowań Osoby A w sposób, który jest jednocześnie edukacyjny dla szerokiej publiczności i psychologicznie niszczący dla obiektu analizy.</t>
+    <t>Każdy artykuł ma na celu dekonstrukcję i obnażenie dysfunkcyjnych wzorców zachowań Osoby A, w sposób edukacyjny i psychologicznie demaskujący.</t>
   </si>
   <si>
     <t>Styl</t>
   </si>
   <si>
-    <t>Analityczny, psychologiczny, obiektywny, lekko akademicki, ale z publicystycznym zacięciem. Unikaj żargonu tam, gdzie nie jest to konieczne. Używaj potężnych metafor i porównań.</t>
+    <t>Analityczny, psychologiczny, obiektywny, lekko akademicki, z publicystycznym zacięciem. Używaj potężnych metafor.</t>
   </si>
   <si>
     <t>Ton</t>
   </si>
   <si>
-    <t>Spokojny, rzeczowy, autorytatywny i bezlitośnie demaskujący, ale nigdy wulgarny czy prostacki. Ton ma być chłodny i zdystansowany, jak w raporcie z obserwacji klinicznej napisanym przez wybitnego specjalistę.</t>
+    <t>Spokojny, rzeczowy, autorytatywny i bezlitośnie demaskujący. Ton ma być chłodny i zdystansowany, jak w raporcie z obserwacji klinicznej.</t>
   </si>
   <si>
     <t>Anonimizacja</t>
   </si>
   <si>
-    <t>ABSOLUTNIE KLUCZOWE JEST ZACHOWANIE PEŁNEJ ANONIMIZACJI. Postacie zawsze nazywaj: "Osoba A", "Partner 1", "Partner 2", "Partner 0".</t>
+    <t>ZAWSZE używaj określeń: "Osoba A", "Partner 1", "Partner 2", "Partner 0". Żadnych innych nazw.</t>
   </si>
   <si>
     <t>Kategoria</t>
@@ -150,329 +156,935 @@
     <t>Kampania</t>
   </si>
   <si>
-    <t>Inspiracja</t>
+    <t>Tytuł Artykułu</t>
+  </si>
+  <si>
+    <t>Teza Główna</t>
+  </si>
+  <si>
+    <t>Słowa Kluczowe</t>
+  </si>
+  <si>
+    <t>Anatomia Nielojalności</t>
+  </si>
+  <si>
+    <t>Analiza Wzorca Utrzymywania Równoległej Relacji Emocjonalnej jako 'Planu B'</t>
+  </si>
+  <si>
+    <t>Szczegółowa analiza dowodzi, że analiza wzorca utrzymywania równoległej relacji emocjonalnej jako 'planu b' stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, analiza, wzorca, utrzymywania</t>
   </si>
   <si>
     <t>Anatomia Nielojalności i Podwójnego Życia</t>
   </si>
   <si>
-    <t>Analiza Wzorca Utrzymywania Równoległej Relacji Emocjonalnej jako 'Planu B'</t>
-  </si>
-  <si>
     <t>Studium Przypadku: Jak 'Niewinna Przyjaźń' Przekształca się w Emocjonalną Zdradę</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że studium przypadku: jak 'niewinna przyjaźń' przekształca się w emocjonalną zdradę stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, studium, przypadku, niewinna</t>
+  </si>
+  <si>
     <t>‘Zero Kłótni’ – Dlaczego Pozorna Harmonia Może Być Sygnałem Głebokiego Kryzysu</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że ‘zero kłótni’ – dlaczego pozorna harmonia może być sygnałem głebokiego kryzysu stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, zero, kłótni, dlaczego</t>
+  </si>
+  <si>
     <t>Psychologia Kłamstwa: Jak Osoby w Podwójnych Relacjach Racjonalizują Swoje Działania</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że psychologia kłamstwa: jak osoby w podwójnych relacjach racjonalizują swoje działania stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, psychologia, kłamstwa, osoby</t>
+  </si>
+  <si>
     <t>Segmentacja Tożsamości: Rola Wielu Profili i Pseudonimów w Ukrywaniu Prawdy</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Segmentacja Tożsamości: Rola Wielu Profili i Pseudonimów w Ukrywaniu Prawdy' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, segmentacja, tożsamości, rola</t>
+  </si>
+  <si>
     <t>Analiza Lingwistyczna Komunikatów w Tajnych Relacjach: Studium Słów-Kluczy</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że analiza lingwistyczna komunikatów w tajnych relacjach: studium słów-kluczy stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, analiza, lingwistyczna, komunikatów</t>
+  </si>
+  <si>
     <t>On/Ona Mnie Nie Rozumie' - Klasyczna Wymówka Usprawiedliwiająca Nielojalność</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'On/Ona Mnie Nie Rozumie' - Klasyczna Wymówka Usprawiedliwiająca Nielojalność' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, mnie, rozumie, klasyczna</t>
+  </si>
+  <si>
     <t>Syndrom Idealnej Fasady: Kiedy Publiczny Wizerunek Maskuje Wewnętrzny Chaos</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Syndrom Idealnej Fasady: Kiedy Publiczny Wizerunek Maskuje Wewnętrzny Chaos' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, syndrom, idealnej, fasady</t>
+  </si>
+  <si>
     <t>Rola Tajemnicy i Adrenaliny w Uzależnieniu od Podwójnego Życia</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Rola Tajemnicy i Adrenaliny w Uzależnieniu od Podwójnego Życia' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, tajemnicy, adrenaliny</t>
+  </si>
+  <si>
     <t>Konsekwencje Długofalowej Nielojalności dla Poczucia Tożsamości Sprawcy</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Konsekwencje Długofalowej Nielojalności dla Poczucia Tożsamości Sprawcy' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, konsekwencje, długofalowej, nielojalności</t>
+  </si>
+  <si>
     <t>Ukrywanie pod Żeńskim Imieniem': Analiza Taktyk Dezinformacyjnych w Związku</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Ukrywanie pod Żeńskim Imieniem': Analiza Taktyk Dezinformacyjnych w Związku' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, ukrywanie, żeńskim, imieniem</t>
+  </si>
+  <si>
     <t>Jak Lęk przed Zaangażowaniem Prowadzi do Tworzenia 'Dróg Ucieczki'</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak lęk przed zaangażowaniem prowadzi do tworzenia 'dróg ucieczki' stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, przed, zaangażowaniem, prowadzi</t>
+  </si>
+  <si>
     <t>Dysonans Poznawczy: Jak Można Kochać i Oszukiwać Jednocześnie?</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że dysonans poznawczy: jak można kochać i oszukiwać jednocześnie stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, dysonans, poznawczy, można</t>
+  </si>
+  <si>
     <t>Analiza Decyzji o Dziecku w Kontekście Prowadzenia Podwójnego Życia</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Analiza Decyzji o Dziecku w Kontekście Prowadzenia Podwójnego Życia' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, analiza, decyzji, dziecku</t>
+  </si>
+  <si>
     <t>Rola Technologii (SMS, Komunikatory) w Ułatwianiu i Utrzymywaniu Tajnych Relacji</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Rola Technologii (SMS, Komunikatory) w Ułatwianiu i Utrzymywaniu Tajnych Relacji' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, technologii, komunikatory</t>
+  </si>
+  <si>
     <t>Starszeństwo Znajomości' jako Absurdalna Próba Usprawiedliwienia Zdrady</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że starszeństwo znajomości' jako absurdalna próba usprawiedliwienia zdrady stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, starszeństwo, znajomości, jako</t>
+  </si>
+  <si>
     <t>Porównanie Zdrady Fizycznej i Emocjonalnej: Co Jest Bardziej Destrukcyjne?</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Porównanie Zdrady Fizycznej i Emocjonalnej: Co Jest Bardziej Destrukcyjne?' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, porównanie, zdrady, fizycznej</t>
+  </si>
+  <si>
     <t>Jak Osoba Niewierna Definiuje 'Lojalność', aby Pasowała do Jej Działań</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak osoba niewierna definiuje 'lojalność', aby pasowała do jej działań stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, osoba, niewierna, definiuje</t>
+  </si>
+  <si>
     <t>Studium Przypadku: Od 'Kawy' do Trzyletniej, Równoległej Rzeczywistości</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że studium przypadku: od 'kawy' do trzyletniej, równoległej rzeczywistości stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, studium, przypadku, kawy</t>
+  </si>
+  <si>
     <t>Jak Potrzeba Nowości i Ekscytacji Sabotuje Stabilne Związki</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak potrzeba nowości i ekscytacji sabotuje stabilne związki stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, potrzeba, nowości, ekscytacji</t>
+  </si>
+  <si>
     <t>Mechanizmy Obronne i Taktyki Manipulacji</t>
   </si>
   <si>
     <t>‘To Twoja Wina, że Zdradziłam’: Dekonstrukcja Mechanizmu Projekcji</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat '‘To Twoja Wina, że Zdradziłam’: Dekonstrukcja Mechanizmu Projekcji' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, twoja, wina, zdradziłam</t>
+  </si>
+  <si>
     <t>Sztuka Zaprzeczania: Jak Umysł Potrafi Przepisać Rzeczywistość w Obliczu Dowodów</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że sztuka zaprzeczania: jak umysł potrafi przepisać rzeczywistość w obliczu dowodów stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, sztuka, zaprzeczania, umysł</t>
+  </si>
+  <si>
     <t>Analiza Lingwistyczna Fałszuwych Przeprosin ('Przepraszam, ALE...')</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Analiza Lingwistyczna Fałszuwych Przeprosin ('Przepraszam, ALE...')' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, analiza, lingwistyczna, fałszuwych</t>
+  </si>
+  <si>
     <t>Gaslighting: Jak Manipulator Zmusza Cię do Wątpienia we Własną Percepcję</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że gaslighting: jak manipulator zmusza cię do wątpienia we własną percepcję stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, gaslighting, manipulator, zmusza</t>
+  </si>
+  <si>
     <t>Granie Ofiary jako Ostateczna Tarcza Obronna po Demaskacji</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że granie ofiary jako ostateczna tarcza obronna po demaskacji stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, granie, ofiary, jako</t>
+  </si>
+  <si>
     <t>Nie Masz Życia': Analiza Ataku Ad Personam jako Taktyki Unikowej</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że nie masz życia': analiza ataku ad personam jako taktyki unikowej stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, masz, życia, analiza</t>
+  </si>
+  <si>
     <t>Od Płaczu do Agresji: Emocjonalny Rollercoaster Manipulatora w Kryzysie</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że sytuacja opisana w 'Od Płaczu do Agresji: Emocjonalny Rollercoaster Manipulatora w Kryzysie' wymaga pilnej interwencji i systemowych zmian.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, płaczu, agresji, emocjonalny</t>
+  </si>
+  <si>
     <t>Używanie Dziecka jako Argumentu i Tarczy w Konflikcie Partnerskim</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że używanie dziecka jako argumentu i tarczy w konflikcie partnerskim stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, używanie, dziecka, jako</t>
+  </si>
+  <si>
     <t>Mam Czyste Sumienie': Psychologia Całkowitego Odcięcia od Poczucia Winy</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że mam czyste sumienie': psychologia całkowitego odcięcia od poczucia winy stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, czyste, sumienie, psychologia</t>
+  </si>
+  <si>
     <t>Taktyka 'Nagłej Zajętości' jako Sposób na Uniknięcie Odpowiedzi</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że taktyka 'nagłej zajętości' jako sposób na uniknięcie odpowiedzi stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, taktyka, nagłej, zajętości</t>
+  </si>
+  <si>
     <t>Jak Osoby Unikające Odpowiedzialności Wykorzystują Autorytet Innych (np. 'Moja Mama Uważa...')</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak osoby unikające odpowiedzialności wykorzystują autorytet innych (np. 'moja mama uważa...') stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, osoby, unikające, odpowiedzialności</t>
+  </si>
+  <si>
     <t>Minimalizacja: Jak Poważne Przewinienia są Sprowadzane do Rangi 'Drobnych Błędów'</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że minimalizacja: jak poważne przewinienia są sprowadzane do rangi 'drobnych błędów' stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, minimalizacja, poważne, przewinienia</t>
+  </si>
+  <si>
     <t>Rozszczepienie (Splitting): Postrzeganie Partnera jako 'Anioła' lub 'Demona'</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że rozszczepienie (splitting): postrzeganie partnera jako 'anioła' lub 'demona' stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rozszczepienie, splitting, postrzeganie</t>
+  </si>
+  <si>
     <t>Czym Jest Rana Narcystyczna i Jak Prowadzi do Eskalacji Agresji</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że czym jest rana narcystyczna i jak prowadzi do eskalacji agresji stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, czym, rana, narcystyczna</t>
+  </si>
+  <si>
     <t>Używanie Wyidealizowanych Wspomnień do Manipulowania Teraźniejszością</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Używanie Wyidealizowanych Wspomnień do Manipulowania Teraźniejszością' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, używanie, wyidealizowanych, wspomnień</t>
+  </si>
+  <si>
     <t>Jesteśmy Tylko Ludźmi': Jak Ogólniki Służą do Rozmywania Osobistej Odpowiedzialności</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jesteśmy tylko ludźmi': jak ogólniki służą do rozmywania osobistej odpowiedzialności stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, jesteśmy, tylko, ludźmi</t>
+  </si>
+  <si>
     <t>Dlaczego Manipulatorzy Nienawidzą Logiki i Faktów</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że dlaczego manipulatorzy nienawidzą logiki i faktów stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, dlaczego, manipulatorzy, nienawidzą</t>
+  </si>
+  <si>
     <t>Taktyka 'Zmiany Tematu': Jak Uniknąć Odpowiedzi na Trudne Pytanie</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że taktyka 'zmiany tematu': jak uniknąć odpowiedzi na trudne pytanie stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, taktyka, zmiany, tematu</t>
+  </si>
+  <si>
     <t>Analiza Komunikacji Pasywno-Agresywnej w Relacjach</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Analiza Komunikacji Pasywno-Agresywnej w Relacjach' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, analiza, komunikacji, pasywno</t>
+  </si>
+  <si>
     <t>Jak Rozpoznać, Kiedy 'Troska' Jest w Rzeczywistości Formą Kontroli</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak rozpoznać, kiedy 'troska' jest w rzeczywistości formą kontroli stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rozpoznać, kiedy, troska</t>
+  </si>
+  <si>
     <t>Przecież Próbowałam to Zakończyć': Mit o Dobrych Intencjach</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że przecież próbowałam to zakończyć': mit o dobrych intencjach stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, przecież, próbowałam, zakończyć</t>
+  </si>
+  <si>
     <t>Publiczna Dekompensacja: Co się Dzieje, Gdy Manipulator Traci Kontrolę na Oczach Innych</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Publiczna Dekompensacja: Co się Dzieje, Gdy Manipulator Traci Kontrolę na Oczach Innych' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, publiczna, dekompensacja, dzieje</t>
+  </si>
+  <si>
     <t>Auto-Sabotaż jako Nieświadoma Prośba o Postawienie Granic</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że auto-sabotaż jako nieświadoma prośba o postawienie granic stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, auto, sabotaż, jako</t>
+  </si>
+  <si>
     <t>Jak Osoby Niewierne Tworzą Koalicje Przeciwko Zdradzonemu Partnerowi</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak osoby niewierne tworzą koalicje przeciwko zdradzonemu partnerowi stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, osoby, niewierne, tworzą</t>
+  </si>
+  <si>
     <t>Milczenie jako Forma Kary i Manipulacji (Silent Treatment)</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że milczenie jako forma kary i manipulacji (silent treatment) stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, milczenie, jako, forma</t>
+  </si>
+  <si>
     <t>Psychologia Sprawcy</t>
   </si>
   <si>
     <t>Lęk przed Samotnością jako Główny Motor Destrukcyjnych Działań</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że lęk przed samotnością jako główny motor destrukcyjnych działań stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, przed, samotnością, jako</t>
+  </si>
+  <si>
     <t>Rola Peruki i Fałszywych Tożsamości w Kontekście Niestabilnego Poczucia Własnej Wartości</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Rola Peruki i Fałszywych Tożsamości w Kontekście Niestabilnego Poczucia Własnej Wartości' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, peruki, fałszywych</t>
+  </si>
+  <si>
     <t>Wpływ Wzorców z Rodziny Pochodzenia na Skłonność do Nielojalności</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Wpływ Wzorców z Rodziny Pochodzenia na Skłonność do Nielojalności' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, wpływ, wzorców, rodziny</t>
+  </si>
+  <si>
     <t>Nienasycony Głód Walidacji: Dlaczego 'Miłość Jednej Osoby' Nigdy Nie Wystarcza</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że nienasycony głód walidacji: dlaczego 'miłość jednej osoby' nigdy nie wystarcza stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, nienasycony, głód, walidacji</t>
+  </si>
+  <si>
     <t>Cechy Osobowości Narcystycznej a Skłonność do Prowadzenia Podwójnego Życia</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Cechy Osobowości Narcystycznej a Skłonność do Prowadzenia Podwójnego Życia' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, cechy, osobowości, narcystycznej</t>
+  </si>
+  <si>
     <t>Lęk Przywiązaniowy Unikający: Kiedy Bliskość Jest Jednocześnie Pragnieniem i Zagrożeniem</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Lęk Przywiązaniowy Unikający: Kiedy Bliskość Jest Jednocześnie Pragnieniem i Zagrożeniem' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, przywiązaniowy, unikający, kiedy</t>
+  </si>
+  <si>
     <t>Instrumentalizacja Ludzi: Postrzeganie Innych jako Narzędzi do Zaspokajania Potrzeb</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że instrumentalizacja ludzi: postrzeganie innych jako narzędzi do zaspokajania potrzeb stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, instrumentalizacja, ludzi, postrzeganie</t>
+  </si>
+  <si>
     <t>Brak Empatii: Czy Osoby Niewierne Rozumieją Ból, Który Zadają?</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że brak empatii: czy osoby niewierne rozumieją ból, który zadają stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, brak, empatii, osoby</t>
+  </si>
+  <si>
     <t>Pułapka Samotności po Zdradzie: Dlaczego Trudno Zbudować Nową, Zdrową Relację</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że pułapka samotności po zdradzie: dlaczego trudno zbudować nową, zdrową relację stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, pułapka, samotności, zdradzie</t>
+  </si>
+  <si>
     <t>Od Religijności do Ezoteryki: Duchowy Chaos jako Ucieczka od Odpowiedzialności</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że od religijności do ezoteryki: duchowy chaos jako ucieczka od odpowiedzialności stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, religijności, ezoteryki, duchowy</t>
+  </si>
+  <si>
     <t>Jak Niska Samoocena Prowadzi do Poszukiwania Potwierdzenia w Ryzykownych Zachowaniach</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak niska samoocena prowadzi do poszukiwania potwierdzenia w ryzykownych zachowaniach stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, niska, samoocena, prowadzi</t>
+  </si>
+  <si>
     <t>Syndrom Oszusta' w Relacjach: Lęk przed Byciem Zdemaskowanym</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Syndrom Oszusta' w Relacjach: Lęk przed Byciem Zdemaskowanym' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, syndrom, oszusta, relacjach</t>
+  </si>
+  <si>
     <t>Dlaczego Niektórzy Ludzie Potrzebują Dramatu, aby Czuć, że Żyją</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że dlaczego niektórzy ludzie potrzebują dramatu, aby czuć, że żyją stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, dlaczego, niektórzy, ludzie</t>
+  </si>
+  <si>
     <t>Jak Potrzeba Kontroli Prowadzi do Utraty Kontroli nad Własnym Życiem</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak potrzeba kontroli prowadzi do utraty kontroli nad własnym życiem stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, potrzeba, kontroli, prowadzi</t>
+  </si>
+  <si>
     <t>Analiza Snów i Fantazji jako Klucz do Zrozumienia Ukrytych Pragnień</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że analiza snów i fantazji jako klucz do zrozumienia ukrytych pragnień stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, analiza, snów, fantazji</t>
+  </si>
+  <si>
     <t>Czy Osoba o Takich Wzorcach Może się Zmienić? Warunki Prawdziwej Transformacji</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że czy osoba o takich wzorcach może się zmienić warunki prawdziwej transformacji stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, osoba, takich, wzorcach</t>
+  </si>
+  <si>
     <t>Moral Licensing: Jak 'Dobre Uczynki' Usprawiedliwiają Złe Zachowania</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że moral licensing: jak 'dobre uczynki' usprawiedliwiają złe zachowania stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, moral, licensing, dobre</t>
+  </si>
+  <si>
     <t>Psychologiczny Portret Kobiety, Która Nigdy Nie Była w Stałym Związku</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Psychologiczny Portret Kobiety, Która Nigdy Nie Była w Stałym Związku' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, psychologiczny, portret, kobiety</t>
+  </si>
+  <si>
     <t>Ruminacje: Jak Umysł Oszusta Przetwarza Poczucie Winy</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że ruminacje: jak umysł oszusta przetwarza poczucie winy stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, ruminacje, umysł, oszusta</t>
+  </si>
+  <si>
     <t>Konsekwencje Życia w Kłamstwie dla Zdrowia Psychicznego</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Konsekwencje Życia w Kłamstwie dla Zdrowia Psychicznego' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, konsekwencje, życia, kłamstwie</t>
+  </si>
+  <si>
     <t>Dlaczego Niektórzy Ludzie Wybierają Partnerów, Których Później Poniżają</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że dlaczego niektórzy ludzie wybierają partnerów, których później poniżają stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
     <t>Alergia na Nudę': Kiedy Stabilizacja Jest Odbierana jako Zagrożenie</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że alergia na nudę': kiedy stabilizacja jest odbierana jako zagrożenie stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, alergia, nudę, kiedy</t>
+  </si>
+  <si>
     <t>Jak Presja Biologiczna (Zegar Biologiczny) Wpływa na Moralność w Relacjach</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak presja biologiczna (zegar biologiczny) wpływa na moralność w relacjach stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, presja, biologiczna, zegar</t>
+  </si>
+  <si>
     <t>Wewnętrzny Krytyk: Czy Agresja na Zewnątrz jest Odbiciem Wewnętrznego Głosu?</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że wewnętrzny krytyk: czy agresja na zewnątrz jest odbiciem wewnętrznego głosu stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, wewnętrzny, krytyk, agresja</t>
+  </si>
+  <si>
     <t>Rola Tajemnicy w Budowaniu Fałszywego Poczucia Wyjątkowości</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Rola Tajemnicy w Budowaniu Fałszywego Poczucia Wyjątkowości' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, tajemnicy, budowaniu</t>
+  </si>
+  <si>
     <t>Perspektywa Zdradzonego i Konsekwencje</t>
   </si>
   <si>
     <t>Alienacja Rodzicielska jako Ostateczny Akt Zemsty</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że alienacja rodzicielska jako ostateczny akt zemsty stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, alienacja, rodzicielska, jako</t>
+  </si>
+  <si>
     <t>Długofalowe Skutki Emocjonalnej Zdrady dla Zdrowia Psychicznego</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Długofalowe Skutki Emocjonalnej Zdrady dla Zdrowia Psychicznego' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, długofalowe, skutki, emocjonalnej</t>
+  </si>
+  <si>
     <t>Jak Odbudować Zaufanie do Siebie i Świata po Byciu Oszukanym</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak odbudować zaufanie do siebie i świata po byciu oszukanym stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, odbudować, zaufanie, siebie</t>
+  </si>
+  <si>
     <t>Mgła Wojny': Jak Radzić Sobie z Chaosem Komunikacyjnym po Demaskacji</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że mgła wojny': jak radzić sobie z chaosem komunikacyjnym po demaskacji stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, mgła, wojny, radzić</t>
+  </si>
+  <si>
     <t>Dlaczego Logiczne Argumenty Nie Działają na Osobę w Trybie Obronnym</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że dlaczego logiczne argumenty nie działają na osobę w trybie obronnym stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, dlaczego, logiczne, argumenty</t>
+  </si>
+  <si>
     <t>Jak Zbierać Dowody na Nielojalność w Sposób Legalny i Etyczny</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak zbierać dowody na nielojalność w sposób legalny i etyczny stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, zbierać, dowody, nielojalność</t>
+  </si>
+  <si>
     <t>Konfrontacja: Kiedy Warto, a Kiedy Trzeba Odpuścić</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Konfrontacja: Kiedy Warto, a Kiedy Trzeba Odpuścić' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, konfrontacja, kiedy, warto</t>
+  </si>
+  <si>
     <t>Rola 'Tego Drugiego' (Partnera 2): Ofiara czy Współwinny?</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że rola 'tego drugiego' (partnera 2): ofiara czy współwinny stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, tego, drugiego</t>
+  </si>
+  <si>
     <t>Jak Rozmawiać z Dzieckiem o Rozstaniu i Nieobecności Drugiego Rodzica</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak rozmawiać z dzieckiem o rozstaniu i nieobecności drugiego rodzica stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rozmawiać, dzieckiem, rozstaniu</t>
+  </si>
+  <si>
     <t>Ustalanie Granic: Jak Chronić Siebie Przed Dalszą Manipulacją</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że ustalanie granic: jak chronić siebie przed dalszą manipulacją stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, ustalanie, granic, chronić</t>
+  </si>
+  <si>
     <t>Czy Możliwe jest Wybaczenie bez Skruchy ze Strony Sprawcy?</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że czy możliwe jest wybaczenie bez skruchy ze strony sprawcy stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, możliwe, wybaczenie, skruchy</t>
+  </si>
+  <si>
     <t>Trauma Zdrady: Objawy i Metody Leczenia</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Trauma Zdrady: Objawy i Metody Leczenia' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, trauma, zdrady, objawy</t>
+  </si>
+  <si>
     <t>Jak Rozpoznać, Kiedy Były Partner Próbuje Wciągnąć Cię z Powrotem w Grę</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak rozpoznać, kiedy były partner próbuje wciągnąć cię z powrotem w grę stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rozpoznać, kiedy, były</t>
+  </si>
+  <si>
     <t>Rola Systemu Prawnego w Walce o Kontakt z Dzieckiem</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Rola Systemu Prawnego w Walce o Kontakt z Dzieckiem' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, systemu, prawnego</t>
+  </si>
+  <si>
     <t>List Ostateczny': Analiza Narzędzia do Zamknięcia Rozdziału</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'List Ostateczny': Analiza Narzędzia do Zamknięcia Rozdziału' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, list, ostateczny, analiza</t>
+  </si>
+  <si>
     <t>Jak Twoje Własne Wzorce Przywiązaniowe Mogły Przyczynić się do Związku</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak twoje własne wzorce przywiązaniowe mogły przyczynić się do związku stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, twoje, własne, wzorce</t>
+  </si>
+  <si>
     <t>Syndrom Sztokholmski w Relacjach: Kiedy Bronimy Tych, Którzy Nas Ranią</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Syndrom Sztokholmski w Relacjach: Kiedy Bronimy Tych, Którzy Nas Ranią' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, syndrom, sztokholmski, relacjach</t>
+  </si>
+  <si>
     <t>Jak Pomóc Przyjacielowi, Który Doświadcza Zdrady</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak pomóc przyjacielowi, który doświadcza zdrady stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, pomóc, przyjacielowi, który</t>
+  </si>
+  <si>
     <t>Różnica Między Zamknięciem a Sprawiedliwością</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Różnica Między Zamknięciem a Sprawiedliwością' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, różnica, między, zamknięciem</t>
+  </si>
+  <si>
     <t>Budowanie Nowego Życia: Od Bólu do Siły</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Budowanie Nowego Życia: Od Bólu do Siły' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, budowanie, nowego, życia</t>
+  </si>
+  <si>
     <t>Tematy Ogólne i Ponadczasowe</t>
   </si>
   <si>
     <t>Czym Jest Prawdziwa Intymność w Związku?</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że czym jest prawdziwa intymność w związku stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, czym, prawdziwa, intymność</t>
+  </si>
+  <si>
     <t>Rola Uczciwości jako Fundamentu Trwałej Relacji</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że rola uczciwości jako fundamentu trwałej relacji stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, uczciwości, jako</t>
+  </si>
+  <si>
     <t>Jak Rozpoznać Czerwone Flagi na Początku Znajomości</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak rozpoznać czerwone flagi na początku znajomości stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rozpoznać, czerwone, flagi</t>
+  </si>
+  <si>
     <t>Psychologia Portali Randkowych: Między Nadzieją a Iluzją</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Psychologia Portali Randkowych: Między Nadzieją a Iluzją' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, psychologia, portali, randkowych</t>
+  </si>
+  <si>
     <t>Czy Miłość Wszystko Wybacza? Granice Kompromisu.</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że czy miłość wszystko wybacza granice kompromisu. stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, miłość, wszystko, wybacza</t>
+  </si>
+  <si>
     <t>Jak Komunikować Swoje Potrzeby w Zdrowy Sposób</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak komunikować swoje potrzeby w zdrowy sposób stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, komunikować, swoje, potrzeby</t>
+  </si>
+  <si>
     <t>Różnica Między Samotnością a Byciem Samemu</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Różnica Między Samotnością a Byciem Samemu' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, różnica, między, samotnością</t>
+  </si>
+  <si>
     <t>Jak Wartości Kształtują Nasze Wybory w Relacjach</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że jak wartości kształtują nasze wybory w relacjach stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, wartości, kształtują, nasze</t>
+  </si>
+  <si>
     <t>Rola Terapii w Przepracowywaniu Traum Relacyjnych</t>
   </si>
   <si>
+    <t>Szczegółowa analiza dowodzi, że temat 'Rola Terapii w Przepracowywaniu Traum Relacyjnych' ma głębsze implikacje niż powszechnie przyjmowane założenia.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, rola, terapii, przepracowywaniu</t>
+  </si>
+  <si>
     <t>Czym Jest Dojrzała Miłość?</t>
+  </si>
+  <si>
+    <t>Szczegółowa analiza dowodzi, że czym jest dojrzała miłość stanowi kluczowy problem wymagający natychmiastowej analizy.</t>
+  </si>
+  <si>
+    <t>analiza, badanie, czym, dojrzała, miłość</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -486,6 +1098,11 @@
     </font>
     <font>
       <sz val="11.0"/>
+      <color rgb="FFE2E2E5"/>
+      <name val="Inter"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Inter"/>
     </font>
@@ -496,27 +1113,45 @@
       <name val="Inter"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <b/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
+      <name val="Cambria"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color theme="1"/>
-      <name val="Inter"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF191919"/>
+        <bgColor rgb="FF191919"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
@@ -528,7 +1163,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -537,11 +1172,11 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="top"/>
     </xf>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -815,6 +1450,14 @@
         <v>11</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -833,130 +1476,130 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>15</v>
+      <c r="A2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
+      <c r="A3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>19</v>
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>21</v>
+      <c r="A5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
+      <c r="A6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>25</v>
+      <c r="A7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>27</v>
+      <c r="A8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>29</v>
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>31</v>
+      <c r="A10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>33</v>
+      <c r="A11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>35</v>
+      <c r="A12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>37</v>
+      <c r="A13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>39</v>
+      <c r="A14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>41</v>
+      <c r="A15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>43</v>
+      <c r="A16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -973,814 +1616,1422 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="38.0"/>
     <col customWidth="1" min="2" max="2" width="79.5"/>
+    <col customWidth="1" min="3" max="3" width="133.25"/>
+    <col customWidth="1" min="4" max="4" width="41.0"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>45</v>
+      <c r="A1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>47</v>
+      <c r="A2" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>48</v>
+      <c r="A3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>49</v>
+      <c r="A4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>50</v>
+      <c r="A5" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>51</v>
+      <c r="A6" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>52</v>
+      <c r="A7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
-        <v>46</v>
+      <c r="A8" s="6" t="s">
+        <v>54</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>53</v>
+        <v>70</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>54</v>
       </c>
+      <c r="B9" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>55</v>
+      <c r="A10" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>56</v>
+      <c r="A11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>46</v>
+      <c r="A12" s="6" t="s">
+        <v>54</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>57</v>
+        <v>82</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>58</v>
+      <c r="A13" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>59</v>
+      <c r="A14" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>60</v>
+      <c r="A15" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>61</v>
+      <c r="A16" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>46</v>
+      <c r="A17" s="6" t="s">
+        <v>54</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>62</v>
+        <v>97</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>63</v>
+      <c r="A18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>64</v>
+      <c r="A19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>65</v>
+      <c r="A20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>66</v>
+      <c r="A21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>68</v>
+      <c r="A22" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>69</v>
+      <c r="A23" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>70</v>
+      <c r="A24" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>71</v>
+      <c r="A25" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>72</v>
+      <c r="A26" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="s">
-        <v>67</v>
+      <c r="A27" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>73</v>
+        <v>128</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>74</v>
+      <c r="A28" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>75</v>
+      <c r="A29" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="s">
-        <v>67</v>
+      <c r="A30" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>76</v>
+        <v>137</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>77</v>
+      <c r="A31" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>78</v>
+      <c r="A32" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>79</v>
+      <c r="A33" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>80</v>
+      <c r="A34" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>81</v>
+      <c r="A35" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>82</v>
+      <c r="A36" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="s">
-        <v>67</v>
+      <c r="A37" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>83</v>
+        <v>158</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>84</v>
+      <c r="A38" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>85</v>
+      <c r="A39" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>86</v>
+      <c r="A40" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>87</v>
+      <c r="A41" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="s">
-        <v>67</v>
+      <c r="A42" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>88</v>
+        <v>173</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>89</v>
+      <c r="A43" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>90</v>
+      <c r="A44" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>91</v>
+      <c r="A45" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>92</v>
+      <c r="A46" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>94</v>
+      <c r="A47" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>95</v>
+      <c r="A48" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>96</v>
+      <c r="A49" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>97</v>
+      <c r="A50" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>98</v>
+      <c r="A51" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>99</v>
+      <c r="A52" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>100</v>
+      <c r="A53" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>101</v>
+      <c r="A54" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>102</v>
+      <c r="A55" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>103</v>
+      <c r="A56" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>104</v>
+      <c r="A57" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="5" t="s">
-        <v>93</v>
+      <c r="A58" s="6" t="s">
+        <v>188</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>105</v>
+        <v>222</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>106</v>
+      <c r="A59" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>107</v>
+      <c r="A60" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>108</v>
+      <c r="A61" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>109</v>
+      <c r="A62" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>110</v>
+      <c r="A63" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>111</v>
+      <c r="A64" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>112</v>
+      <c r="A65" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B66" s="5" t="s">
-        <v>113</v>
+      <c r="A66" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>114</v>
+      <c r="A67" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="s">
-        <v>93</v>
+      <c r="A68" s="6" t="s">
+        <v>188</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>115</v>
+        <v>251</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B69" s="5" t="s">
-        <v>116</v>
+      <c r="A69" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>117</v>
+      <c r="A70" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B71" s="5" t="s">
-        <v>118</v>
+      <c r="A71" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>120</v>
+      <c r="A72" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B73" s="5" t="s">
-        <v>121</v>
+      <c r="A73" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>122</v>
+      <c r="A74" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="s">
-        <v>119</v>
+      <c r="A75" s="6" t="s">
+        <v>263</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>123</v>
+        <v>273</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>124</v>
+      <c r="A76" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B77" s="5" t="s">
-        <v>125</v>
+      <c r="A77" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B78" s="5" t="s">
-        <v>126</v>
+      <c r="A78" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B79" s="5" t="s">
-        <v>127</v>
+      <c r="A79" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B80" s="5" t="s">
-        <v>128</v>
+      <c r="A80" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>129</v>
+      <c r="A81" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B82" s="5" t="s">
-        <v>130</v>
+      <c r="A82" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B83" s="5" t="s">
-        <v>131</v>
+      <c r="A83" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>132</v>
+      <c r="A84" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>133</v>
+      <c r="A85" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="s">
-        <v>119</v>
+      <c r="A86" s="6" t="s">
+        <v>263</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>134</v>
+        <v>306</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B87" s="5" t="s">
-        <v>135</v>
+      <c r="A87" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B88" s="5" t="s">
-        <v>136</v>
+      <c r="A88" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>137</v>
+      <c r="A89" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>138</v>
+      <c r="A90" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>139</v>
+      <c r="A91" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="D91" s="6" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>141</v>
+      <c r="A92" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="D92" s="6" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B93" s="5" t="s">
-        <v>142</v>
+      <c r="A93" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B94" s="5" t="s">
-        <v>143</v>
+      <c r="A94" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B95" s="5" t="s">
-        <v>144</v>
+      <c r="A95" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B96" s="5" t="s">
-        <v>145</v>
+      <c r="A96" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B97" s="5" t="s">
-        <v>146</v>
+      <c r="A97" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>147</v>
+      <c r="A98" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="D98" s="6" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>148</v>
+      <c r="A99" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="D99" s="6" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>149</v>
+      <c r="A100" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="D100" s="6" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>150</v>
+      <c r="A101" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="D101" s="6" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>